<commit_message>
Add Saratoga Surrender Site and confirmed 2026 US250 programming
Added the Saratoga Surrender Site as an 11th stop with Trumbull bas-relief
detail. Updated Saratoga NHP practical info with confirmed 2026 events:
Victory Season Living History Weekend (Oct 10-11), Turning Point Symposium
(May 2), Knox Noble Train recreation, and saratoga250.com as event source.

https://claude.ai/code/session_0187xe2kC3K88cb7LNSbwWDY
</commit_message>
<xml_diff>
--- a/outputs/upstate-listings-master.xlsx
+++ b/outputs/upstate-listings-master.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -829,12 +829,12 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>upstate-schuyler-house-saratoga</t>
+          <t>upstate-saratoga-surrender-site</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Schuyler House (Saratoga NHP)</t>
+          <t>Saratoga Surrender Site</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -854,27 +854,27 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>43.1003</t>
+          <t>43.0940</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>-73.5831</t>
+          <t>-73.5850</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Burgoyne burned it on his retreat — Schuyler rebuilt it within a year</t>
+          <t>The field where 5,895 British soldiers laid down their arms — and changed the world</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>After Burgoyne retreated north from the battlefield, he burned Schuyler's country estate. Schuyler rebuilt this house within a year — a declaration that the Schuylers weren't leaving. The site sits near the surrender field where Burgoyne's army laid down their arms.</t>
+          <t>On October 17, 1777, Burgoyne's army surrendered here — the first time an entire British army had capitulated in history. The 19-acre site holds a granite wall, a bronze bas-relief of Trumbull's painting, and a landscape that hasn't changed much since 1777.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>When Burgoyne's retreating army burned Philip Schuyler's country estate in October 1777, it was an act of spite by a losing general. Schuyler rebuilt this house within a year on the same foundation — equal parts stubbornness and strategy. The house sits a few miles from the field where Burgoyne surrendered 5,895 men, and its reconstruction was as much a political statement as a personal one: the Schuylers owned this valley, and they intended to stay. The interior reflects Schuyler's wealth and the domestic life of one of the revolution's architects. Don't miss: the view from the back of the house toward the Hudson — the same view Schuyler saw when he chose to rebuild on scorched ground.</t>
+          <t>On October 17, 1777, British General John Burgoyne surrendered 5,895 men in this field along the Hudson River — the first time an entire British army had capitulated in history. Within months, France recognized the United States, and a colonial rebellion became a global conflict. The 19-acre site is quiet now: a granite wall faces the river, and a bronze bas-relief reproduces John Trumbull's painting The Surrender of General Burgoyne, the original of which hangs in the U.S. Capitol Rotunda. The landscape is remarkably unchanged since 1777. Don't miss: the bronze bas-relief of Trumbull's Surrender of General Burgoyne — then compare it to the original next time you're in the Capitol.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -899,7 +899,11 @@
           <t>https://www.nps.gov/sara</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>https://saratoga250.com</t>
+        </is>
+      </c>
       <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr"/>
       <c r="T4" s="2" t="inlineStr"/>
@@ -910,7 +914,7 @@
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>{"Business Category": "Cultural Heritage", "Business Type": "Historic House", "County": ["Saratoga County"], "Region": ["Capital-Saratoga Region"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Guided Tour"]}</t>
+          <t>{"Business Category": "Experience", "Business Type": "National Park", "County": ["Saratoga County"], "Region": ["Capital-Saratoga Region"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Scenic Views"]}</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -927,17 +931,17 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>upstate-saratoga-monument</t>
+          <t>upstate-schuyler-house-saratoga</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Saratoga Monument</t>
+          <t>Schuyler House (Saratoga NHP)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>1 Burgoyne Street</t>
+          <t>Route 4</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -952,27 +956,27 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>43.0997</t>
+          <t>43.1003</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>-73.5814</t>
+          <t>-73.5831</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Four niches for four generals — one has been empty since 1883</t>
+          <t>Burgoyne burned it on his retreat — Schuyler rebuilt it within a year</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The 155-foot obelisk has four niches for the American generals at Saratoga. Three hold statues: Schuyler, Gates, Morgan. The fourth — Arnold's — has been empty since the monument was dedicated in 1883. You can climb the interior staircase for a view across the entire campaign landscape.</t>
+          <t>After Burgoyne retreated north from the battlefield, he burned Schuyler's country estate. Schuyler rebuilt this house within a year — a declaration that the Schuylers weren't leaving. The site sits near the surrender field where Burgoyne's army laid down their arms.</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Dedicated in 1883, this 155-foot obelisk in the center of Schuylerville commemorates the American victory at Saratoga with four niches — one for each commanding general. Three hold bronze statues of Schuyler, Gates, and Morgan. The fourth niche, meant for Benedict Arnold, stands deliberately empty. Arnold's charge at Bemis Heights broke the British line and arguably won the battle, but his subsequent treason made him unmemorable in bronze. The empty niche is the most eloquent commentary on treason and heroism in American public art. Climb the interior staircase to the top for a panoramic view of the Hudson Valley that maps the entire 1777 campaign. Don't miss: the empty fourth niche — stand in front of it and consider what it means that a nation would carve a space for a hero it couldn't name.</t>
+          <t>When Burgoyne's retreating army burned Philip Schuyler's country estate in October 1777, it was an act of spite by a losing general. Schuyler rebuilt this house within a year on the same foundation — equal parts stubbornness and strategy. The house sits a few miles from the field where Burgoyne surrendered 5,895 men, and its reconstruction was as much a political statement as a personal one: the Schuylers owned this valley, and they intended to stay. The interior reflects Schuyler's wealth and the domestic life of one of the revolution's architects. Don't miss: the view from the back of the house toward the Hudson — the same view Schuyler saw when he chose to rebuild on scorched ground.</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -1008,7 +1012,7 @@
       <c r="Y5" s="3" t="inlineStr"/>
       <c r="Z5" s="3" t="inlineStr">
         <is>
-          <t>{"Business Category": "Experience", "Business Type": "Battlefield", "County": ["Saratoga County"], "Region": ["Capital-Saratoga Region"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Scenic Views"]}</t>
+          <t>{"Business Category": "Cultural Heritage", "Business Type": "Historic House", "County": ["Saratoga County"], "Region": ["Capital-Saratoga Region"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Guided Tour"]}</t>
         </is>
       </c>
       <c r="AA5" s="3" t="inlineStr">
@@ -1025,52 +1029,52 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>upstate-fort-stanwix-national-monument</t>
+          <t>upstate-saratoga-monument</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fort Stanwix National Monument</t>
+          <t>Saratoga Monument</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>112 East Park Street</t>
+          <t>1 Burgoyne Street</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Rome</t>
+          <t>Schuylerville</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Oneida County</t>
+          <t>Saratoga County</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>43.2106</t>
+          <t>43.0997</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>-75.4557</t>
+          <t>-73.5814</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>550 men held this fort for 21 days — and stopped a British army cold</t>
+          <t>Four niches for four generals — one has been empty since 1883</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Colonel Peter Gansevoort held this frontier fort against a British force three times his size for 21 days in August 1777. The western arm of Burgoyne's strategy to split the colonies died here, at a bend in the Mohawk River that most travelers drive past.</t>
+          <t>The 155-foot obelisk has four niches for the American generals at Saratoga. Three hold statues: Schuyler, Gates, Morgan. The fourth — Arnold's — has been empty since the monument was dedicated in 1883. You can climb the interior staircase for a view across the entire campaign landscape.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>In August 1777, Colonel Peter Gansevoort held this frontier fort with 550 men against Barry St. Leger's force of 1,700 British regulars, Loyalists, and Haudenosaunee allies for 21 days — long enough for Benedict Arnold's relief column to force a retreat. The western arm of Burgoyne's plan to split the colonies in two died here, at a bend in the Mohawk River. The NPS has reconstructed the fort to its 1758 appearance; uniformed rangers know the siege hour by hour. But the fort's significance stretches beyond 1777: the 1768 Treaty of Fort Stanwix, signed here, ceded vast Haudenosaunee territories and set the stage for every conflict that followed. Don't miss: the 1768 Treaty exhibit — the document that redrew the boundary between colonial settlement and Haudenosaunee territory.</t>
+          <t>Dedicated in 1883, this 155-foot obelisk in the center of Schuylerville commemorates the American victory at Saratoga with four niches — one for each commanding general. Three hold bronze statues of Schuyler, Gates, and Morgan. The fourth niche, meant for Benedict Arnold, stands deliberately empty. Arnold's charge at Bemis Heights broke the British line and arguably won the battle, but his subsequent treason made him unmemorable in bronze. The empty niche is the most eloquent commentary on treason and heroism in American public art. Climb the interior staircase to the top for a panoramic view of the Hudson Valley that maps the entire 1777 campaign. Don't miss: the empty fourth niche — stand in front of it and consider what it means that a nation would carve a space for a hero it couldn't name.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1080,7 +1084,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>13440</t>
+          <t>12871</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -1092,7 +1096,7 @@
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/fost</t>
+          <t>https://www.nps.gov/sara</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
@@ -1106,7 +1110,7 @@
       <c r="Y6" s="2" t="inlineStr"/>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>{"Business Category": "Experience", "Business Type": "National Park", "County": ["Oneida County"], "Region": ["Mohawk Valley"], "Trail": ["Revolutionary War Sites", "Haudenosaunee Heritage Trail"], "Experience": ["History &amp; Heritage", "Living History", "Guided Tour", "Educational", "Family-Friendly"]}</t>
+          <t>{"Business Category": "Experience", "Business Type": "Battlefield", "County": ["Saratoga County"], "Region": ["Capital-Saratoga Region"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Scenic Views"]}</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1123,22 +1127,22 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>upstate-oriskany-battlefield-state-historic-site</t>
+          <t>upstate-fort-stanwix-national-monument</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Oriskany Battlefield State Historic Site</t>
+          <t>Fort Stanwix National Monument</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>7801 State Route 69</t>
+          <t>112 East Park Street</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Oriskany</t>
+          <t>Rome</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1148,27 +1152,27 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>43.1570</t>
+          <t>43.2106</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>-75.3730</t>
+          <t>-75.4557</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>The bloodiest battle of the Revolution by casualty rate — and the day the Confederacy fractured</t>
+          <t>550 men held this fort for 21 days — and stopped a British army cold</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>On August 6, 1777, General Herkimer's relief column walked into an ambush in this ravine. The fighting was hand-to-hand. Oneida fought Mohawk. When it was over, the Haudenosaunee Confederacy's centuries-old unity was broken along lines that never fully healed.</t>
+          <t>Colonel Peter Gansevoort held this frontier fort against a British force three times his size for 21 days in August 1777. The western arm of Burgoyne's strategy to split the colonies died here, at a bend in the Mohawk River that most travelers drive past.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>On August 6, 1777, a relief column of 800 Oneida warriors and Tryon County militia marching to break the siege of Fort Stanwix walked into an ambush in a ravine beside Oriskany Creek. The fighting was hand-to-hand. Neighbors killed neighbors. Oneida warriors fought Mohawk warriors in what was effectively a Haudenosaunee civil war. General Nicholas Herkimer took a musket ball through the knee, had his men prop him against a beech tree, lit his pipe, and directed the battle for six hours while bleeding to death. The casualty rate was the highest of any Revolutionary War battle. The monument on the hill marks where Herkimer sat. Don't miss: stand at the edge of the ravine where the ambush began — the terrain explains the battle better than any exhibit.</t>
+          <t>In August 1777, Colonel Peter Gansevoort held this frontier fort with 550 men against Barry St. Leger's force of 1,700 British regulars, Loyalists, and Haudenosaunee allies for 21 days — long enough for Benedict Arnold's relief column to force a retreat. The western arm of Burgoyne's plan to split the colonies in two died here, at a bend in the Mohawk River. The NPS has reconstructed the fort to its 1758 appearance; uniformed rangers know the siege hour by hour. But the fort's significance stretches beyond 1777: the 1768 Treaty of Fort Stanwix, signed here, ceded vast Haudenosaunee territories and set the stage for every conflict that followed. Don't miss: the 1768 Treaty exhibit — the document that redrew the boundary between colonial settlement and Haudenosaunee territory.</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1178,7 +1182,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>13424</t>
+          <t>13440</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1190,7 +1194,7 @@
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>https://parks.ny.gov/historic-sites/oriskany-battlefield</t>
+          <t>https://www.nps.gov/fost</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr"/>
@@ -1204,7 +1208,7 @@
       <c r="Y7" s="3" t="inlineStr"/>
       <c r="Z7" s="3" t="inlineStr">
         <is>
-          <t>{"Business Category": "Experience", "Business Type": "Battlefield", "County": ["Oneida County"], "Region": ["Mohawk Valley"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Indigenous Culture"]}</t>
+          <t>{"Business Category": "Experience", "Business Type": "National Park", "County": ["Oneida County"], "Region": ["Mohawk Valley"], "Trail": ["Revolutionary War Sites", "Haudenosaunee Heritage Trail"], "Experience": ["History &amp; Heritage", "Living History", "Guided Tour", "Educational", "Family-Friendly"]}</t>
         </is>
       </c>
       <c r="AA7" s="3" t="inlineStr">
@@ -1221,52 +1225,52 @@
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>upstate-herkimer-home-state-historic-site</t>
+          <t>upstate-oriskany-battlefield-state-historic-site</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Herkimer Home State Historic Site</t>
+          <t>Oriskany Battlefield State Historic Site</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>200 State Route 169</t>
+          <t>7801 State Route 69</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Little Falls</t>
+          <t>Oriskany</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Herkimer County</t>
+          <t>Oneida County</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>43.0120</t>
+          <t>43.1570</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>-74.8840</t>
+          <t>-75.3730</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>The general who commanded from a beech tree — and died reading his Bible in German</t>
+          <t>The bloodiest battle of the Revolution by casualty rate — and the day the Confederacy fractured</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Herkimer was carried from Oriskany to this house on the Mohawk River, where a botched amputation killed him ten days later. He reportedly read his Bible aloud in German — his first language — as he died. The house is a fine Georgian brick home in a county of frame farmhouses.</t>
+          <t>On August 6, 1777, General Herkimer's relief column walked into an ambush in this ravine. The fighting was hand-to-hand. Oneida fought Mohawk. When it was over, the Haudenosaunee Confederacy's centuries-old unity was broken along lines that never fully healed.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Herkimer was the wealthiest man in the Mohawk Valley and chose to march anyway. After taking a musket ball through the knee at Oriskany, he was carried to this Georgian brick house on the Mohawk River. A Continental Army surgeon amputated his shattered leg ten days after the battle. The amputation went wrong. Herkimer bled to death on August 16, 1777, reportedly reading his Bible aloud in German — his first language — to his family. The house stands in a landscape of frame farmhouses, a reminder of Herkimer's status and his sacrifice. Little Falls (population 4,500) is a Mohawk Valley mill town that rewards a slow drive through. Don't miss: the room where Herkimer died — the family Bible and bed placement are based on period accounts.</t>
+          <t>On August 6, 1777, a relief column of 800 Oneida warriors and Tryon County militia marching to break the siege of Fort Stanwix walked into an ambush in a ravine beside Oriskany Creek. The fighting was hand-to-hand. Neighbors killed neighbors. Oneida warriors fought Mohawk warriors in what was effectively a Haudenosaunee civil war. General Nicholas Herkimer took a musket ball through the knee, had his men prop him against a beech tree, lit his pipe, and directed the battle for six hours while bleeding to death. The casualty rate was the highest of any Revolutionary War battle. The monument on the hill marks where Herkimer sat. Don't miss: stand at the edge of the ravine where the ambush began — the terrain explains the battle better than any exhibit.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1276,7 +1280,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>13365</t>
+          <t>13424</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1288,14 +1292,10 @@
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>https://parks.ny.gov/historic-sites/herkimer-home</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>https://mohawkvalleyhistory.com</t>
-        </is>
-      </c>
+          <t>https://parks.ny.gov/historic-sites/oriskany-battlefield</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
@@ -1306,7 +1306,7 @@
       <c r="Y8" s="2" t="inlineStr"/>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>{"Business Category": "Cultural Heritage", "Business Type": "State Historic Site", "County": ["Herkimer County"], "Region": ["Mohawk Valley"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Guided Tour"]}</t>
+          <t>{"Business Category": "Experience", "Business Type": "Battlefield", "County": ["Oneida County"], "Region": ["Mohawk Valley"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Indigenous Culture"]}</t>
         </is>
       </c>
       <c r="AA8" s="2" t="inlineStr">
@@ -1323,52 +1323,52 @@
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>upstate-old-stone-fort-museum</t>
+          <t>upstate-herkimer-home-state-historic-site</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Old Stone Fort Museum</t>
+          <t>Herkimer Home State Historic Site</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>145 Fort Road</t>
+          <t>200 State Route 169</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Schoharie</t>
+          <t>Little Falls</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Schoharie County</t>
+          <t>Herkimer County</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>42.6660</t>
+          <t>43.0120</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>-74.3120</t>
+          <t>-74.8840</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>A 1772 church fortified for war — holding the Palatine German story no one else tells</t>
+          <t>The general who commanded from a beech tree — and died reading his Bible in German</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Schoharie is a county seat of 1,200 people. This 1772 Reformed church, fortified during the Revolution and raided by Joseph Brant in 1780, holds the story of the Palatine German migration of 1710 — 3,000 Rhineland refugees who became the backbone of the Mohawk Valley militia.</t>
+          <t>Nicholas Herkimer was carried from Oriskany to this house on the Mohawk River, where a botched amputation killed him ten days later. He reportedly read his Bible aloud in German — his first language — as he died. The house is a fine Georgian brick home in a county of frame farmhouses.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Schoharie is a county seat of 1,200 people, and the Old Stone Fort Museum on the edge of town tells a story you'll find nowhere else. In 1710, three thousand Palatine German refugees from the Rhineland settled the Schoharie and Mohawk Valleys. Their descendants became the backbone of the frontier militia that fought at Oriskany and defended the valley throughout the Revolution. This 1772 Reformed church was fortified during the war and survived a 1780 raid by Joseph Brant and Sir John Johnson. The collection inside is local, personal, and irreplaceable: ledgers, tools, family Bibles in German script, and a genealogy archive that traces Palatine families back to 1710. Don't miss: the Palatine German genealogy collection — if your family came through the Schoharie Valley, the records here go back three centuries.</t>
+          <t>Nicholas Herkimer was the wealthiest man in the Mohawk Valley and chose to march anyway. After taking a musket ball through the knee at Oriskany, he was carried to this Georgian brick house on the Mohawk River. A Continental Army surgeon amputated his shattered leg ten days after the battle. The amputation went wrong. Herkimer bled to death on August 16, 1777, reportedly reading his Bible aloud in German — his first language — to his family. The house stands in a landscape of frame farmhouses, a reminder of Herkimer's status and his sacrifice. Little Falls (population 4,500) is a Mohawk Valley mill town that rewards a slow drive through. Don't miss: the room where Herkimer died — the family Bible and bed placement are based on period accounts.</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>12157</t>
+          <t>13365</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1390,10 +1390,14 @@
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>https://www.theoldstonefort.org</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="inlineStr"/>
+          <t>https://parks.ny.gov/historic-sites/herkimer-home</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>https://mohawkvalleyhistory.com</t>
+        </is>
+      </c>
       <c r="R9" s="3" t="inlineStr"/>
       <c r="S9" s="3" t="inlineStr"/>
       <c r="T9" s="3" t="inlineStr"/>
@@ -1404,7 +1408,7 @@
       <c r="Y9" s="3" t="inlineStr"/>
       <c r="Z9" s="3" t="inlineStr">
         <is>
-          <t>{"Business Category": "Cultural Heritage", "Business Type": "Museum", "County": ["Schoharie County"], "Region": ["Capital-Saratoga Region"], "Trail": ["Revolutionary War Sites", "Path Through History"], "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Educational"]}</t>
+          <t>{"Business Category": "Cultural Heritage", "Business Type": "State Historic Site", "County": ["Herkimer County"], "Region": ["Mohawk Valley"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Guided Tour"]}</t>
         </is>
       </c>
       <c r="AA9" s="3" t="inlineStr">
@@ -1421,52 +1425,52 @@
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>upstate-crown-point-state-historic-site</t>
+          <t>upstate-old-stone-fort-museum</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Crown Point State Historic Site</t>
+          <t>Old Stone Fort Museum</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>739 Bridge Road</t>
+          <t>145 Fort Road</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Crown Point</t>
+          <t>Schoharie</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Essex County</t>
+          <t>Schoharie County</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>43.9430</t>
+          <t>42.6660</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>-73.4250</t>
+          <t>-74.3120</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Ruins of two great forts on a limestone promontory — and almost nobody comes here</t>
+          <t>A 1772 church fortified for war — holding the Palatine German story no one else tells</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Two days after Allen took Ticonderoga, Seth Warner captured Crown Point — and 111 more cannons. The ruins of the massive 1759 British fort and the earlier French Fort St. Frederic form one of the most impressive military landscapes in North America. Crown Point (population 2,000) is an RTN destination.</t>
+          <t>Schoharie is a county seat of 1,200 people. This 1772 Reformed church, fortified during the Revolution and raided by Joseph Brant in 1780, holds the story of the Palatine German migration of 1710 — 3,000 Rhineland refugees who became the backbone of the Mohawk Valley militia.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Two days after Ethan Allen captured Fort Ticonderoga, Seth Warner took Crown Point and its 111 additional cannons. The ruins here are older and more imposing than Ticonderoga's: the massive stone walls of the 1759 British fort — built to hold 4,000 troops — and the remains of the earlier French Fort St. Frederic form one of the most impressive colonial military landscapes in North America. Crown Point (population 2,000) sits on a limestone promontory jutting into Lake Champlain, and on a clear day the view reaches into Vermont and Canada. Almost nobody comes here, which is exactly why you should. The scale of the crumbling walls against the lake is the most dramatic physical remnant of the colonial wars in New York. Don't miss: the ruins of Fort St. Frederic — the French fortification whose walls crumble directly into Lake Champlain.</t>
+          <t>Schoharie is a county seat of 1,200 people, and the Old Stone Fort Museum on the edge of town tells a story you'll find nowhere else. In 1710, three thousand Palatine German refugees from the Rhineland settled the Schoharie and Mohawk Valleys. Their descendants became the backbone of the frontier militia that fought at Oriskany and defended the valley throughout the Revolution. This 1772 Reformed church was fortified during the war and survived a 1780 raid by Joseph Brant and Sir John Johnson. The collection inside is local, personal, and irreplaceable: ledgers, tools, family Bibles in German script, and a genealogy archive that traces Palatine families back to 1710. Don't miss: the Palatine German genealogy collection — if your family came through the Schoharie Valley, the records here go back three centuries.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1476,7 +1480,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>12928</t>
+          <t>12157</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1488,14 +1492,10 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>https://parks.ny.gov/historic-sites/crown-point</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>https://visitadirondacks.com</t>
-        </is>
-      </c>
+          <t>https://www.theoldstonefort.org</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
@@ -1506,7 +1506,7 @@
       <c r="Y10" s="2" t="inlineStr"/>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>{"Business Category": "Experience", "Business Type": "Fort", "County": ["Essex County"], "Region": ["Adirondacks"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Scenic Views", "Hiking"]}</t>
+          <t>{"Business Category": "Cultural Heritage", "Business Type": "Museum", "County": ["Schoharie County"], "Region": ["Capital-Saratoga Region"], "Trail": ["Revolutionary War Sites", "Path Through History"], "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Educational"]}</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
@@ -1523,22 +1523,22 @@
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>upstate-fort-ticonderoga</t>
+          <t>upstate-crown-point-state-historic-site</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Fort Ticonderoga</t>
+          <t>Crown Point State Historic Site</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>102 Fort Ti Road</t>
+          <t>739 Bridge Road</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Ticonderoga</t>
+          <t>Crown Point</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1548,27 +1548,27 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>43.8391</t>
+          <t>43.9430</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>-73.3894</t>
+          <t>-73.4250</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>America's first offensive victory — 59 cannons that ended the siege of Boston</t>
+          <t>Ruins of two great forts on a limestone promontory — and almost nobody comes here</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Ethan Allen arrived with 83 men and no artillery plan. He left with the cannons that Henry Knox dragged 300 miles on ox sleds to end the siege of Boston. Fort Ticonderoga's REAL TIME REVOLUTION program — immersive and running through 2027 — is built for the 250th anniversary.</t>
+          <t>Two days after Allen took Ticonderoga, Seth Warner captured Crown Point — and 111 more cannons. The ruins of the massive 1759 British fort and the earlier French Fort St. Frederic form one of the most impressive military landscapes in North America. Crown Point (population 2,000) is an RTN destination.</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>On the night of May 10, 1775, Ethan Allen and 83 Green Mountain Boys crossed Lake Champlain in the dark and captured the British garrison in what one soldier called 'a confused melee of shouting.' It was America's first offensive military victory, and it mattered less for the symbolism than for the 59 cannons Henry Knox dragged 300 miles on ox sleds to Dorchester Heights the following winter, ending the siege of Boston. The fort has been restored to its 18th-century appearance by the Mars family since 1908 and is the most thoroughly interpreted colonial military site in the country. The King's Garden, between the fort and the lake, is one of the most beautiful cultivated spaces in the Adirondacks. Don't miss: the view from the ramparts north across Lake Champlain to Mount Defiance — the high ground the British seized in 1777 to force the American evacuation.</t>
+          <t>Two days after Ethan Allen captured Fort Ticonderoga, Seth Warner took Crown Point and its 111 additional cannons. The ruins here are older and more imposing than Ticonderoga's: the massive stone walls of the 1759 British fort — built to hold 4,000 troops — and the remains of the earlier French Fort St. Frederic form one of the most impressive colonial military landscapes in North America. Crown Point (population 2,000) sits on a limestone promontory jutting into Lake Champlain, and on a clear day the view reaches into Vermont and Canada. Almost nobody comes here, which is exactly why you should. The scale of the crumbling walls against the lake is the most dramatic physical remnant of the colonial wars in New York. Don't miss: the ruins of Fort St. Frederic — the French fortification whose walls crumble directly into Lake Champlain.</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>12883</t>
+          <t>12928</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -1590,12 +1590,12 @@
       <c r="O11" s="3" t="inlineStr"/>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>https://www.fortticonderoga.org</t>
+          <t>https://parks.ny.gov/historic-sites/crown-point</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>https://america250.org</t>
+          <t>https://visitadirondacks.com</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr"/>
@@ -1608,15 +1608,117 @@
       <c r="Y11" s="3" t="inlineStr"/>
       <c r="Z11" s="3" t="inlineStr">
         <is>
+          <t>{"Business Category": "Experience", "Business Type": "Fort", "County": ["Essex County"], "Region": ["Adirondacks"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Self-Guided Tour", "Scenic Views", "Hiking"]}</t>
+        </is>
+      </c>
+      <c r="AA11" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AB11" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>upstate-fort-ticonderoga</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Fort Ticonderoga</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>102 Fort Ti Road</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Ticonderoga</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Essex County</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>43.8391</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>-73.3894</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>America's first offensive victory — 59 cannons that ended the siege of Boston</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Ethan Allen arrived with 83 men and no artillery plan. He left with the cannons that Henry Knox dragged 300 miles on ox sleds to end the siege of Boston. Fort Ticonderoga's REAL TIME REVOLUTION program — immersive and running through 2027 — is built for the 250th anniversary.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>On the night of May 10, 1775, Ethan Allen and 83 Green Mountain Boys crossed Lake Champlain in the dark and captured the British garrison in what one soldier called 'a confused melee of shouting.' It was America's first offensive military victory, and it mattered less for the symbolism than for the 59 cannons Henry Knox dragged 300 miles on ox sleds to Dorchester Heights the following winter, ending the siege of Boston. The fort has been restored to its 18th-century appearance by the Mars family since 1908 and is the most thoroughly interpreted colonial military site in the country. The King's Garden, between the fort and the lake, is one of the most beautiful cultivated spaces in the Adirondacks. Don't miss: the view from the ramparts north across Lake Champlain to Mount Defiance — the high ground the British seized in 1777 to force the American evacuation.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>12883</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fortticonderoga.org</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>https://america250.org</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="inlineStr"/>
+      <c r="X12" s="2" t="inlineStr"/>
+      <c r="Y12" s="2" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
           <t>{"Business Category": "Experience", "Business Type": "Fort", "County": ["Essex County"], "Region": ["Adirondacks"], "Trail": "Revolutionary War Sites", "Experience": ["History &amp; Heritage", "Living History", "Guided Tour", "Scenic Views", "Educational", "Family-Friendly"]}</t>
         </is>
       </c>
-      <c r="AA11" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="AB11" s="3" t="inlineStr">
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>